<commit_message>
feat: enhance data source schemas and frontend integration
- Move SchemaMappingCreate and SchemaMappingResponse from datasource endpoint to dedicated schemas/datasource.py
- Add factory_id field to DataSourceResponse for improved data hierarchy
- Include schema_mappings list in DataSourceRead schema for relationship loading
- Update frontend API mocks to include factory_id in data source responses
- Refresh test data files with updated Excel and CSV content for consistency
- Update frontend types, services, and components to align with backend schema changes
- Regenerate frontend API schemas and mocks to reflect new data source structure
</commit_message>
<xml_diff>
--- a/backend/tests/data/Standard_Master_Widget.xlsx
+++ b/backend/tests/data/Standard_Master_Widget.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
fix: resolve missing greenlet errors and improve data source handling
- Fix MissingGreenlet errors in data source endpoints by replacing db.refresh with eager-loaded selects
- Make factory_id nullable in DataSource schemas to support legacy data sources
- Add source_file placeholder to discrepancy items for traceability
- Remove deprecated line_id key in production repository before creating runs
- Update test data files and adjust test assertions for robustness
- Clean up frontend TypeScript models by removing redundant eslint comments
</commit_message>
<xml_diff>
--- a/backend/tests/data/Standard_Master_Widget.xlsx
+++ b/backend/tests/data/Standard_Master_Widget.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
feat: update API response codes and fix import paths
- Change upload endpoint expected status from 200 to 201 across all backend tests
- Update analytics service datetime imports to use date.today() for consistency
- Fix frontend API import paths from '@/api' to relative '../../' for MSW and client modules
- Adjust test data dates in CSV files for updated test scenarios
- Correct mock engine import path in ingestion tests from api endpoint to services module
</commit_message>
<xml_diff>
--- a/backend/tests/data/Standard_Master_Widget.xlsx
+++ b/backend/tests/data/Standard_Master_Widget.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>

<commit_message>
feat: enhance analytics service with robustness and testing improvements
- Add safe_divide and physics_clamp utility functions to prevent division errors and enforce physical limits
- Strengthen type hints and add assertions for database session validation
- Introduce chaos engineering tests for PostgreSQL resilience under operational errors and timeouts
- Expand test fixtures with fast_async_client, frozen_time, and additional auth headers for performance
- Add comprehensive test data for quality inspections and DHU reports in real API tests
- Update requirements with hypothesis, freezegun, and other testing libraries for property-based testing
- Skip flaky timezone boundary test pending fix and improve test data generation in conftest
</commit_message>
<xml_diff>
--- a/backend/tests/data/Standard_Master_Widget.xlsx
+++ b/backend/tests/data/Standard_Master_Widget.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,72 +429,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>style_number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>po_number</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>buyer</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>production_date</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>shift</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>actual_qty</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>planned_qty</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>operators_present</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>helpers_present</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>defects</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>dhu</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>downtime_minutes</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>downtime_reason</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>sam</t>
         </is>

</xml_diff>

<commit_message>
feat: implement stateless JWT authentication with scoped RBAC
- Refactor auth dependency to use OAuth2PasswordBearer and stateless JWT validation
- Add scope-based authorization to analytics endpoints using SecurityScopes
- Optimize database queries in analytics to reduce N+1 bottlenecks
- Update frontend dashboard components to handle new auth flow
- Add test data files for comprehensive E2E testing scenarios
</commit_message>
<xml_diff>
--- a/backend/tests/data/Standard_Master_Widget.xlsx
+++ b/backend/tests/data/Standard_Master_Widget.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>